<commit_message>
Update Casestudy to stylized Austrian system
Switch to newest InOutModule
</commit_message>
<xml_diff>
--- a/data/hydroExample/Global_Parameters.xlsx
+++ b/data/hydroExample/Global_Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD9B932-79A3-44F9-B21B-0DA8D023B87B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1489DE12-2AEF-4F70-B23F-E1E17510D66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33915" yWindow="-21810" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Parameters" sheetId="121" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>[h]</t>
   </si>
@@ -138,9 +138,6 @@
     <t>pSolver</t>
   </si>
   <si>
-    <t>highs</t>
-  </si>
-  <si>
     <t>Selected solver</t>
   </si>
   <si>
@@ -193,6 +190,12 @@
   </si>
   <si>
     <t>v0.1.0</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>gurobi</t>
   </si>
 </sst>
 </file>
@@ -837,10 +840,10 @@
     </row>
     <row r="2" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>41</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -880,19 +883,19 @@
         <v>23</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="F5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="G5" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="H5" s="13" t="s">
         <v>27</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -916,7 +919,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>9</v>
@@ -938,7 +941,7 @@
     </row>
     <row r="10" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" s="10"/>
       <c r="E10" s="10"/>
@@ -948,10 +951,10 @@
     </row>
     <row r="11" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
@@ -960,19 +963,19 @@
     </row>
     <row r="12" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" s="9">
         <v>1E-3</v>
       </c>
       <c r="E12" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="15" t="s">
         <v>33</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>34</v>
       </c>
       <c r="H12" s="13">
         <v>1E-3</v>
@@ -985,10 +988,10 @@
     </row>
     <row r="14" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E14" s="11"/>
       <c r="F14" s="11"/>
@@ -996,19 +999,19 @@
     </row>
     <row r="15" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" s="9">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>39</v>
-      </c>
       <c r="G15" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H15" s="13">
         <v>1E-3</v>

</xml_diff>

<commit_message>
Switch to rMIP solve
</commit_message>
<xml_diff>
--- a/data/hydroExample/Global_Parameters.xlsx
+++ b/data/hydroExample/Global_Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1489DE12-2AEF-4F70-B23F-E1E17510D66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8491EB-14F9-43BD-97AA-1A7D9453379D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>[h]</t>
   </si>
@@ -190,9 +190,6 @@
   </si>
   <si>
     <t>v0.1.0</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>gurobi</t>
@@ -883,7 +880,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>24</v>
@@ -919,7 +916,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>9</v>
@@ -1112,18 +1109,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1273,6 +1270,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1284,14 +1289,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>